<commit_message>
A  app/Models/TelegramUser.php A  app/Services/TelegramService.php A  app/Telegram/Commands/StartCommand.php M  config/telegram.php A  database/migrations/2025_01_31_150846_create_telegram_users_table.php M  database/seeders/xlsx/dastan24.02.xlsx M  routes/web.php
</commit_message>
<xml_diff>
--- a/database/seeders/xlsx/dastan24.02.xlsx
+++ b/database/seeders/xlsx/dastan24.02.xlsx
@@ -444,7 +444,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -476,12 +476,6 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF555555"/>
-      <name val="Verdana"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1050,137 +1044,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1223,12 +1217,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1552,7 +1540,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="5.77777777777778" customWidth="1"/>
@@ -1610,13 +1598,13 @@
       <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="25" t="s">
+      <c r="O1" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="25" t="s">
+      <c r="P1" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="27" t="s">
+      <c r="Q1" s="23" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1803,10 +1791,10 @@
       <c r="H6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
       <c r="M6" s="5">
         <v>999999</v>
       </c>
@@ -2008,10 +1996,10 @@
       <c r="H11" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="26"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="22"/>
+      <c r="L11" s="22"/>
       <c r="M11" s="5">
         <v>999999</v>
       </c>
@@ -2049,10 +2037,10 @@
       <c r="H12" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="26"/>
+      <c r="I12" s="22"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="22"/>
+      <c r="L12" s="22"/>
       <c r="M12" s="5">
         <v>999999</v>
       </c>
@@ -2090,10 +2078,10 @@
       <c r="H13" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="26"/>
-      <c r="J13" s="26"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="26"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="22"/>
       <c r="M13" s="5">
         <v>999999</v>
       </c>
@@ -2131,10 +2119,10 @@
       <c r="H14" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="26"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="26"/>
+      <c r="I14" s="22"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="22"/>
+      <c r="L14" s="22"/>
       <c r="M14" s="5">
         <v>999999</v>
       </c>
@@ -2888,82 +2876,6 @@
       <c r="Q32" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:17">
-      <c r="A33" s="12"/>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
-      <c r="L33" s="5"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="5"/>
-      <c r="O33" s="5"/>
-      <c r="P33" s="5"/>
-      <c r="Q33" s="5"/>
-    </row>
-    <row r="34" spans="1:17">
-      <c r="A34" s="12"/>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5"/>
-      <c r="L34" s="5"/>
-      <c r="M34" s="5"/>
-      <c r="N34" s="5"/>
-      <c r="O34" s="5"/>
-      <c r="P34" s="5"/>
-      <c r="Q34" s="5"/>
-    </row>
-    <row r="35" spans="1:17">
-      <c r="A35" s="12"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
-      <c r="L35" s="5"/>
-      <c r="M35" s="5"/>
-      <c r="N35" s="5"/>
-      <c r="O35" s="5"/>
-      <c r="P35" s="5"/>
-      <c r="Q35" s="5"/>
-    </row>
-    <row r="36" spans="1:17">
-      <c r="A36" s="22"/>
-      <c r="B36" s="23"/>
-      <c r="C36" s="23"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="23"/>
-      <c r="G36" s="23"/>
-      <c r="H36" s="23"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="23"/>
-      <c r="K36" s="23"/>
-      <c r="L36" s="23"/>
-      <c r="M36" s="23"/>
-      <c r="N36" s="23"/>
-      <c r="O36" s="23"/>
-      <c r="P36" s="23"/>
-      <c r="Q36" s="23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>